<commit_message>
#15 #14 #13 #12 BOM added.
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_CIM_v1.5/BOM/Client-BOM-OFP_CIM_v1.5.xlsx
+++ b/Design-Files/OFP_CIM_v1.5/BOM/Client-BOM-OFP_CIM_v1.5.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="97">
   <si>
     <t>#</t>
   </si>
@@ -307,13 +307,16 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>This Part Use As Peripheral</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,6 +359,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -472,7 +490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -511,6 +529,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -811,7 +841,7 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1093,28 +1123,30 @@
       <c r="C10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="15">
         <v>3</v>
       </c>
-      <c r="K10" s="9"/>
+      <c r="K10" s="16" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>

</xml_diff>

<commit_message>
#17 CIM and VIM Client BOM Updated.
Connector Change kiye han
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_CIM_v1.5/BOM/Client-BOM-OFP_CIM_v1.5.xlsx
+++ b/Design-Files/OFP_CIM_v1.5/BOM/Client-BOM-OFP_CIM_v1.5.xlsx
@@ -81,9 +81,6 @@
     <t>J2</t>
   </si>
   <si>
-    <t>J3, J4, J5</t>
-  </si>
-  <si>
     <t>LED1, LED2, LED3, LED4, LED5, LED6, LED7, LED8, LED9, LED10, LED11, LED12</t>
   </si>
   <si>
@@ -126,15 +123,9 @@
     <t>DIODE ARR GP 100V 215MA TO-236AB</t>
   </si>
   <si>
-    <t>450V 17.5A 18 Bend -40℃~+105℃ 1 5.08mm 1x18P Green Board end/socket - Open type Push-Pull,P=5.08mm Pluggable System Terminal Block ROHS</t>
-  </si>
-  <si>
     <t>CONN HDR 24POS 0.1 GOLD PCB R/A</t>
   </si>
   <si>
-    <t>450V 17.5A 6 -40℃~+105℃ 1.5 1 14~28 5.08mm 1x6P Green Plug P=5.08mm Pluggable System Terminal Block ROHS</t>
-  </si>
-  <si>
     <t>Emerald 0603 Light Emitting Diodes (LED) ROHS</t>
   </si>
   <si>
@@ -171,9 +162,6 @@
     <t>SOT-23</t>
   </si>
   <si>
-    <t>DB2ER-5.08-18P-GN</t>
-  </si>
-  <si>
     <t>SFH11-PBPC-D12-RA-BK</t>
   </si>
   <si>
@@ -210,9 +198,6 @@
     <t>BAV99,215</t>
   </si>
   <si>
-    <t>DB2EK-5.08-6P-GN-S</t>
-  </si>
-  <si>
     <t>NCD0603G2</t>
   </si>
   <si>
@@ -249,9 +234,6 @@
     <t>Nexperia</t>
   </si>
   <si>
-    <t>DIBO</t>
-  </si>
-  <si>
     <t>Sullins</t>
   </si>
   <si>
@@ -310,6 +292,24 @@
   </si>
   <si>
     <t>This Part Use As Peripheral</t>
+  </si>
+  <si>
+    <t>DB2ERM-5.08-18P-GN</t>
+  </si>
+  <si>
+    <t>DB2EKM-5.08-18P-GN-S</t>
+  </si>
+  <si>
+    <t>320V 20A 18 Bend -40℃~+105℃ 1 5.08mm 1x18P Green Receptacle-Close Screw Fixing Push-Pull,P=5.08mm Pluggable System Terminal Block ROHS</t>
+  </si>
+  <si>
+    <t>DORABO</t>
+  </si>
+  <si>
+    <t>-40℃~+105℃ 2.5 1 14~28 5.08mm 320V 20A 18 1x18P Green Plug Screw Fixing P=5.08mm Pluggable System Terminal Block ROHS</t>
+  </si>
+  <si>
+    <t>J3</t>
   </si>
 </sst>
 </file>
@@ -527,20 +527,20 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -842,6 +842,7 @@
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -853,9 +854,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -869,25 +870,25 @@
         <v>12</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -903,19 +904,19 @@
         <v>13</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="J3" s="7">
         <v>36</v>
@@ -935,19 +936,19 @@
         <v>14</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J4" s="9">
         <v>6</v>
@@ -967,19 +968,19 @@
         <v>15</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="J5" s="7">
         <v>16</v>
@@ -999,19 +1000,19 @@
         <v>16</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J6" s="9">
         <v>13</v>
@@ -1031,19 +1032,19 @@
         <v>17</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J7" s="7">
         <v>18</v>
@@ -1063,19 +1064,19 @@
         <v>18</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1095,19 +1096,19 @@
         <v>19</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1123,29 +1124,29 @@
       <c r="C10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="15" t="s">
+      <c r="D10" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="G10" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="18" t="s">
+      <c r="F10" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="J10" s="15">
-        <v>3</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>96</v>
+      <c r="I10" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" s="14">
+        <v>1</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1158,22 +1159,22 @@
         <v>7</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J11" s="7">
         <v>12</v>
@@ -1190,22 +1191,22 @@
         <v>8</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="J12" s="9">
         <v>30</v>
@@ -1222,22 +1223,22 @@
         <v>8</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="J13" s="7">
         <v>18</v>
@@ -1254,22 +1255,22 @@
         <v>9</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="J14" s="9">
         <v>18</v>
@@ -1286,22 +1287,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="J15" s="7">
         <v>3</v>
@@ -1318,22 +1319,22 @@
         <v>8</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="I16" s="10" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="J16" s="9">
         <v>12</v>
@@ -1350,22 +1351,22 @@
         <v>10</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J17" s="7">
         <v>3</v>
@@ -1382,22 +1383,22 @@
         <v>11</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J18" s="9">
         <v>3</v>

</xml_diff>